<commit_message>
Enterprise Batch Multi-Format Conversion: test-strategy.xlsx
</commit_message>
<xml_diff>
--- a/test-strategy.xlsx
+++ b/test-strategy.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,22 +429,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>User Story ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>

</xml_diff>

<commit_message>
Universal Multi-Format Deployment: test-strategy.xlsx
</commit_message>
<xml_diff>
--- a/test-strategy.xlsx
+++ b/test-strategy.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +28,33 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -51,14 +68,34 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,68 +464,74 @@
   </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>User Story ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Authentication</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>US-001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Login Page</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>US-002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>User Stats</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>